<commit_message>
Fixed version of the 65C64 instruction architecture.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="1320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="1344">
   <si>
     <t xml:space="preserve">Pin number</t>
   </si>
@@ -6040,6 +6040,78 @@
   </si>
   <si>
     <t xml:space="preserve">pul (A, V, W), S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">badd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block subtract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bsub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bcmp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vadd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector subtract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vsub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vcmp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 = Add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 = Subtract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 = Compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 = Add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 = Subtract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 = Compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 = Unused</t>
   </si>
 </sst>
 </file>
@@ -14947,7 +15019,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:M123"/>
+  <dimension ref="A2:M117"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.64"/>
@@ -16921,10 +16993,10 @@
         <v>63</v>
       </c>
       <c r="C74" s="30" t="s">
-        <v>483</v>
+        <v>1320</v>
       </c>
       <c r="D74" s="30" t="s">
-        <v>484</v>
+        <v>1321</v>
       </c>
       <c r="E74" s="111"/>
       <c r="F74" s="111"/>
@@ -16950,23 +17022,26 @@
         <v>64</v>
       </c>
       <c r="C75" s="30" t="s">
-        <v>486</v>
+        <v>1322</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>487</v>
+        <v>1323</v>
       </c>
       <c r="E75" s="111"/>
       <c r="F75" s="111"/>
       <c r="G75" s="30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H75" s="125"/>
       <c r="I75" s="115"/>
       <c r="J75" s="114" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="K75" s="114" t="s">
         <v>471</v>
+      </c>
+      <c r="L75" s="0" t="s">
+        <v>493</v>
       </c>
       <c r="M75" s="103"/>
     </row>
@@ -16977,53 +17052,58 @@
         <v>65</v>
       </c>
       <c r="C76" s="30" t="s">
-        <v>488</v>
+        <v>1324</v>
       </c>
       <c r="D76" s="30" t="s">
-        <v>489</v>
+        <v>1325</v>
       </c>
       <c r="E76" s="111"/>
       <c r="F76" s="111"/>
       <c r="G76" s="30" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H76" s="125"/>
       <c r="I76" s="115"/>
       <c r="J76" s="114" t="s">
-        <v>1290</v>
+        <v>1292</v>
       </c>
       <c r="K76" s="114" t="s">
         <v>471</v>
       </c>
+      <c r="L76" s="0" t="s">
+        <v>497</v>
+      </c>
       <c r="M76" s="103"/>
     </row>
-    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="103"/>
       <c r="B77" s="0" t="n">
         <f aca="false">B76+1</f>
         <v>66</v>
       </c>
       <c r="C77" s="30" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="D77" s="30" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="E77" s="111"/>
       <c r="F77" s="111"/>
       <c r="G77" s="30" t="n">
-        <v>9</v>
-      </c>
-      <c r="H77" s="125"/>
+        <v>12</v>
+      </c>
+      <c r="H77" s="125" t="s">
+        <v>465</v>
+      </c>
       <c r="I77" s="115"/>
       <c r="J77" s="114" t="s">
-        <v>1291</v>
+        <v>1294</v>
       </c>
       <c r="K77" s="114" t="s">
         <v>471</v>
       </c>
       <c r="L77" s="0" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="M77" s="103"/>
     </row>
@@ -17034,26 +17114,26 @@
         <v>67</v>
       </c>
       <c r="C78" s="30" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="D78" s="30" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="E78" s="111"/>
       <c r="F78" s="111"/>
       <c r="G78" s="30" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H78" s="125"/>
       <c r="I78" s="115"/>
       <c r="J78" s="114" t="s">
-        <v>1292</v>
+        <v>1295</v>
       </c>
       <c r="K78" s="114" t="s">
         <v>471</v>
       </c>
       <c r="L78" s="0" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="M78" s="103"/>
     </row>
@@ -17064,85 +17144,84 @@
         <v>68</v>
       </c>
       <c r="C79" s="30" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="D79" s="30" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="E79" s="111"/>
       <c r="F79" s="111"/>
       <c r="G79" s="30" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H79" s="125"/>
       <c r="I79" s="115"/>
       <c r="J79" s="114" t="s">
-        <v>1293</v>
+        <v>1296</v>
       </c>
       <c r="K79" s="114" t="s">
         <v>471</v>
       </c>
       <c r="M79" s="103"/>
     </row>
-    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="103"/>
       <c r="B80" s="0" t="n">
         <f aca="false">B79+1</f>
         <v>69</v>
       </c>
       <c r="C80" s="30" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="D80" s="30" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="E80" s="111"/>
       <c r="F80" s="111"/>
       <c r="G80" s="30" t="n">
-        <v>12</v>
-      </c>
-      <c r="H80" s="125" t="s">
-        <v>465</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H80" s="125"/>
       <c r="I80" s="115"/>
       <c r="J80" s="114" t="s">
-        <v>1294</v>
+        <v>1297</v>
       </c>
       <c r="K80" s="114" t="s">
         <v>471</v>
       </c>
-      <c r="L80" s="0" t="s">
-        <v>503</v>
-      </c>
       <c r="M80" s="103"/>
     </row>
-    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="103"/>
       <c r="B81" s="0" t="n">
         <f aca="false">B80+1</f>
         <v>70</v>
       </c>
       <c r="C81" s="30" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="D81" s="30" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="E81" s="111"/>
-      <c r="F81" s="111"/>
+      <c r="F81" s="111" t="n">
+        <v>3</v>
+      </c>
       <c r="G81" s="30" t="n">
-        <v>13</v>
-      </c>
-      <c r="H81" s="125"/>
+        <v>0</v>
+      </c>
+      <c r="H81" s="125" t="s">
+        <v>465</v>
+      </c>
       <c r="I81" s="115"/>
       <c r="J81" s="114" t="s">
-        <v>1295</v>
+        <v>513</v>
       </c>
       <c r="K81" s="114" t="s">
         <v>471</v>
       </c>
       <c r="L81" s="0" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="M81" s="103"/>
     </row>
@@ -17153,23 +17232,26 @@
         <v>71</v>
       </c>
       <c r="C82" s="30" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="D82" s="30" t="s">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="E82" s="111"/>
       <c r="F82" s="111"/>
       <c r="G82" s="30" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H82" s="125"/>
-      <c r="I82" s="115"/>
+      <c r="I82" s="127"/>
       <c r="J82" s="114" t="s">
-        <v>1296</v>
+        <v>517</v>
       </c>
       <c r="K82" s="114" t="s">
         <v>471</v>
+      </c>
+      <c r="L82" s="0" t="s">
+        <v>518</v>
       </c>
       <c r="M82" s="103"/>
     </row>
@@ -17180,57 +17262,53 @@
         <v>72</v>
       </c>
       <c r="C83" s="30" t="s">
-        <v>509</v>
+        <v>519</v>
       </c>
       <c r="D83" s="30" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="E83" s="111"/>
       <c r="F83" s="111"/>
       <c r="G83" s="30" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H83" s="125"/>
       <c r="I83" s="115"/>
       <c r="J83" s="114" t="s">
-        <v>1297</v>
+        <v>521</v>
       </c>
       <c r="K83" s="114" t="s">
         <v>471</v>
       </c>
+      <c r="L83" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="M83" s="103"/>
     </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="103"/>
       <c r="B84" s="0" t="n">
         <f aca="false">B83+1</f>
         <v>73</v>
       </c>
       <c r="C84" s="30" t="s">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="D84" s="30" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="E84" s="111"/>
-      <c r="F84" s="111" t="n">
+      <c r="F84" s="111"/>
+      <c r="G84" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="G84" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H84" s="125" t="s">
-        <v>465</v>
-      </c>
+      <c r="H84" s="125"/>
       <c r="I84" s="115"/>
       <c r="J84" s="114" t="s">
-        <v>513</v>
+        <v>1274</v>
       </c>
       <c r="K84" s="114" t="s">
         <v>471</v>
-      </c>
-      <c r="L84" s="0" t="s">
-        <v>514</v>
       </c>
       <c r="M84" s="103"/>
     </row>
@@ -17241,26 +17319,23 @@
         <v>74</v>
       </c>
       <c r="C85" s="30" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="D85" s="30" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="E85" s="111"/>
       <c r="F85" s="111"/>
       <c r="G85" s="30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H85" s="125"/>
-      <c r="I85" s="127"/>
+      <c r="I85" s="115"/>
       <c r="J85" s="114" t="s">
-        <v>517</v>
+        <v>1275</v>
       </c>
       <c r="K85" s="114" t="s">
         <v>471</v>
-      </c>
-      <c r="L85" s="0" t="s">
-        <v>518</v>
       </c>
       <c r="M85" s="103"/>
     </row>
@@ -17271,50 +17346,49 @@
         <v>75</v>
       </c>
       <c r="C86" s="30" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="D86" s="30" t="s">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="E86" s="111"/>
       <c r="F86" s="111"/>
       <c r="G86" s="30" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H86" s="125"/>
       <c r="I86" s="115"/>
       <c r="J86" s="114" t="s">
-        <v>521</v>
+        <v>1276</v>
       </c>
       <c r="K86" s="114" t="s">
         <v>471</v>
       </c>
-      <c r="L86" s="0" t="s">
-        <v>522</v>
-      </c>
       <c r="M86" s="103"/>
     </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="103"/>
       <c r="B87" s="0" t="n">
         <f aca="false">B86+1</f>
         <v>76</v>
       </c>
       <c r="C87" s="30" t="s">
-        <v>523</v>
+        <v>1326</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>524</v>
+        <v>1327</v>
       </c>
       <c r="E87" s="111"/>
       <c r="F87" s="111"/>
       <c r="G87" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="H87" s="125"/>
+        <v>6</v>
+      </c>
+      <c r="H87" s="125" t="s">
+        <v>422</v>
+      </c>
       <c r="I87" s="115"/>
       <c r="J87" s="114" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="K87" s="114" t="s">
         <v>471</v>
@@ -17328,20 +17402,20 @@
         <v>77</v>
       </c>
       <c r="C88" s="30" t="s">
-        <v>526</v>
+        <v>1328</v>
       </c>
       <c r="D88" s="30" t="s">
-        <v>527</v>
+        <v>1329</v>
       </c>
       <c r="E88" s="111"/>
       <c r="F88" s="111"/>
       <c r="G88" s="30" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H88" s="125"/>
       <c r="I88" s="115"/>
       <c r="J88" s="114" t="s">
-        <v>1275</v>
+        <v>1279</v>
       </c>
       <c r="K88" s="114" t="s">
         <v>471</v>
@@ -17355,20 +17429,20 @@
         <v>78</v>
       </c>
       <c r="C89" s="30" t="s">
-        <v>529</v>
+        <v>1330</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>530</v>
+        <v>1331</v>
       </c>
       <c r="E89" s="111"/>
       <c r="F89" s="111"/>
       <c r="G89" s="30" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H89" s="125"/>
       <c r="I89" s="115"/>
       <c r="J89" s="114" t="s">
-        <v>1276</v>
+        <v>538</v>
       </c>
       <c r="K89" s="114" t="s">
         <v>471</v>
@@ -17382,25 +17456,28 @@
         <v>79</v>
       </c>
       <c r="C90" s="30" t="s">
-        <v>531</v>
+        <v>545</v>
       </c>
       <c r="D90" s="30" t="s">
-        <v>532</v>
+        <v>546</v>
       </c>
       <c r="E90" s="111"/>
       <c r="F90" s="111"/>
       <c r="G90" s="30" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H90" s="125" t="s">
-        <v>422</v>
+        <v>465</v>
       </c>
       <c r="I90" s="115"/>
       <c r="J90" s="114" t="s">
-        <v>1277</v>
+        <v>513</v>
       </c>
       <c r="K90" s="114" t="s">
         <v>471</v>
+      </c>
+      <c r="L90" s="0" t="s">
+        <v>514</v>
       </c>
       <c r="M90" s="103"/>
     </row>
@@ -17411,20 +17488,20 @@
         <v>80</v>
       </c>
       <c r="C91" s="30" t="s">
-        <v>534</v>
+        <v>547</v>
       </c>
       <c r="D91" s="30" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="E91" s="111"/>
       <c r="F91" s="111"/>
       <c r="G91" s="30" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H91" s="125"/>
       <c r="I91" s="115"/>
       <c r="J91" s="114" t="s">
-        <v>1278</v>
+        <v>521</v>
       </c>
       <c r="K91" s="114" t="s">
         <v>471</v>
@@ -17438,20 +17515,20 @@
         <v>81</v>
       </c>
       <c r="C92" s="30" t="s">
-        <v>536</v>
+        <v>549</v>
       </c>
       <c r="D92" s="30" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="E92" s="111"/>
       <c r="F92" s="111"/>
       <c r="G92" s="30" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H92" s="125"/>
       <c r="I92" s="115"/>
       <c r="J92" s="114" t="s">
-        <v>1279</v>
+        <v>1281</v>
       </c>
       <c r="K92" s="114" t="s">
         <v>471</v>
@@ -17465,20 +17542,20 @@
         <v>82</v>
       </c>
       <c r="C93" s="30" t="s">
-        <v>539</v>
+        <v>551</v>
       </c>
       <c r="D93" s="30" t="s">
-        <v>540</v>
+        <v>552</v>
       </c>
       <c r="E93" s="111"/>
       <c r="F93" s="111"/>
       <c r="G93" s="30" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H93" s="125"/>
       <c r="I93" s="115"/>
       <c r="J93" s="114" t="s">
-        <v>1280</v>
+        <v>1282</v>
       </c>
       <c r="K93" s="114" t="s">
         <v>471</v>
@@ -17492,24 +17569,26 @@
         <v>83</v>
       </c>
       <c r="C94" s="30" t="s">
-        <v>541</v>
+        <v>553</v>
       </c>
       <c r="D94" s="30" t="s">
-        <v>542</v>
-      </c>
-      <c r="E94" s="111"/>
-      <c r="F94" s="111"/>
-      <c r="G94" s="30" t="n">
-        <v>10</v>
-      </c>
-      <c r="H94" s="125"/>
+        <v>1269</v>
+      </c>
+      <c r="E94" s="111" t="n">
+        <v>15</v>
+      </c>
+      <c r="F94" s="121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="128"/>
+      <c r="H94" s="57" t="s">
+        <v>554</v>
+      </c>
       <c r="I94" s="115"/>
       <c r="J94" s="114" t="s">
-        <v>538</v>
-      </c>
-      <c r="K94" s="114" t="s">
-        <v>471</v>
-      </c>
+        <v>555</v>
+      </c>
+      <c r="K94" s="114"/>
       <c r="M94" s="103"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17519,56 +17598,47 @@
         <v>84</v>
       </c>
       <c r="C95" s="30" t="s">
-        <v>543</v>
+        <v>556</v>
       </c>
       <c r="D95" s="30" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="E95" s="111"/>
-      <c r="F95" s="111"/>
-      <c r="G95" s="30" t="n">
-        <v>11</v>
-      </c>
-      <c r="H95" s="125"/>
+      <c r="F95" s="121" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="124"/>
+      <c r="H95" s="57"/>
       <c r="I95" s="115"/>
       <c r="J95" s="114" t="s">
-        <v>538</v>
-      </c>
-      <c r="K95" s="114" t="s">
-        <v>471</v>
-      </c>
+        <v>558</v>
+      </c>
+      <c r="K95" s="114"/>
       <c r="M95" s="103"/>
     </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="103"/>
       <c r="B96" s="0" t="n">
         <f aca="false">B95+1</f>
         <v>85</v>
       </c>
       <c r="C96" s="30" t="s">
-        <v>545</v>
+        <v>559</v>
       </c>
       <c r="D96" s="30" t="s">
-        <v>546</v>
+        <v>560</v>
       </c>
       <c r="E96" s="111"/>
-      <c r="F96" s="111"/>
-      <c r="G96" s="30" t="n">
-        <v>12</v>
-      </c>
-      <c r="H96" s="125" t="s">
-        <v>465</v>
-      </c>
+      <c r="F96" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="G96" s="124"/>
+      <c r="H96" s="57"/>
       <c r="I96" s="115"/>
       <c r="J96" s="114" t="s">
-        <v>513</v>
-      </c>
-      <c r="K96" s="114" t="s">
-        <v>471</v>
-      </c>
-      <c r="L96" s="0" t="s">
-        <v>514</v>
-      </c>
+        <v>561</v>
+      </c>
+      <c r="K96" s="114"/>
       <c r="M96" s="103"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17578,24 +17648,22 @@
         <v>86</v>
       </c>
       <c r="C97" s="30" t="s">
-        <v>547</v>
+        <v>562</v>
       </c>
       <c r="D97" s="30" t="s">
-        <v>548</v>
+        <v>563</v>
       </c>
       <c r="E97" s="111"/>
-      <c r="F97" s="111"/>
-      <c r="G97" s="30" t="n">
-        <v>13</v>
-      </c>
-      <c r="H97" s="125"/>
+      <c r="F97" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="G97" s="124"/>
+      <c r="H97" s="57"/>
       <c r="I97" s="115"/>
       <c r="J97" s="114" t="s">
-        <v>521</v>
-      </c>
-      <c r="K97" s="114" t="s">
-        <v>471</v>
-      </c>
+        <v>564</v>
+      </c>
+      <c r="K97" s="114"/>
       <c r="M97" s="103"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17605,23 +17673,25 @@
         <v>87</v>
       </c>
       <c r="C98" s="30" t="s">
-        <v>549</v>
+        <v>565</v>
       </c>
       <c r="D98" s="30" t="s">
-        <v>550</v>
+        <v>566</v>
       </c>
       <c r="E98" s="111"/>
-      <c r="F98" s="111"/>
-      <c r="G98" s="30" t="n">
-        <v>14</v>
-      </c>
-      <c r="H98" s="125"/>
+      <c r="F98" s="121" t="n">
+        <v>4</v>
+      </c>
+      <c r="G98" s="124"/>
+      <c r="H98" s="57" t="s">
+        <v>328</v>
+      </c>
       <c r="I98" s="115"/>
       <c r="J98" s="114" t="s">
-        <v>1281</v>
+        <v>567</v>
       </c>
       <c r="K98" s="114" t="s">
-        <v>471</v>
+        <v>568</v>
       </c>
       <c r="M98" s="103"/>
     </row>
@@ -17632,24 +17702,22 @@
         <v>88</v>
       </c>
       <c r="C99" s="30" t="s">
-        <v>551</v>
+        <v>569</v>
       </c>
       <c r="D99" s="30" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="E99" s="111"/>
-      <c r="F99" s="111"/>
-      <c r="G99" s="30" t="n">
-        <v>15</v>
-      </c>
-      <c r="H99" s="125"/>
+      <c r="F99" s="121" t="n">
+        <v>5</v>
+      </c>
+      <c r="G99" s="124"/>
+      <c r="H99" s="57"/>
       <c r="I99" s="115"/>
       <c r="J99" s="114" t="s">
-        <v>1282</v>
-      </c>
-      <c r="K99" s="114" t="s">
-        <v>471</v>
-      </c>
+        <v>571</v>
+      </c>
+      <c r="K99" s="114"/>
       <c r="M99" s="103"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17659,380 +17727,222 @@
         <v>89</v>
       </c>
       <c r="C100" s="30" t="s">
-        <v>553</v>
+        <v>572</v>
       </c>
       <c r="D100" s="30" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E100" s="111" t="n">
-        <v>15</v>
-      </c>
+        <v>573</v>
+      </c>
+      <c r="E100" s="111"/>
       <c r="F100" s="121" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="128"/>
-      <c r="H100" s="57" t="s">
-        <v>554</v>
-      </c>
-      <c r="I100" s="115"/>
+        <v>7</v>
+      </c>
+      <c r="G100" s="126"/>
+      <c r="H100" s="57"/>
+      <c r="I100" s="129"/>
       <c r="J100" s="114" t="s">
-        <v>555</v>
-      </c>
-      <c r="K100" s="114"/>
+        <v>574</v>
+      </c>
+      <c r="K100" s="114" t="s">
+        <v>568</v>
+      </c>
       <c r="M100" s="103"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="103"/>
-      <c r="B101" s="0" t="n">
-        <f aca="false">B100+1</f>
-        <v>90</v>
-      </c>
-      <c r="C101" s="30" t="s">
-        <v>556</v>
-      </c>
-      <c r="D101" s="30" t="s">
-        <v>557</v>
-      </c>
-      <c r="E101" s="111"/>
-      <c r="F101" s="121" t="n">
-        <v>1</v>
-      </c>
-      <c r="G101" s="124"/>
-      <c r="H101" s="57"/>
-      <c r="I101" s="115"/>
-      <c r="J101" s="114" t="s">
-        <v>558</v>
-      </c>
-      <c r="K101" s="114"/>
       <c r="M101" s="103"/>
     </row>
-    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="103"/>
-      <c r="B102" s="0" t="n">
-        <f aca="false">B101+1</f>
-        <v>91</v>
-      </c>
-      <c r="C102" s="30" t="s">
-        <v>559</v>
-      </c>
-      <c r="D102" s="30" t="s">
-        <v>560</v>
-      </c>
-      <c r="E102" s="111"/>
-      <c r="F102" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="G102" s="124"/>
-      <c r="H102" s="57"/>
-      <c r="I102" s="115"/>
-      <c r="J102" s="114" t="s">
-        <v>561</v>
-      </c>
-      <c r="K102" s="114"/>
+      <c r="C102" s="130" t="s">
+        <v>575</v>
+      </c>
+      <c r="D102" s="130"/>
+      <c r="E102" s="130"/>
+      <c r="F102" s="130"/>
+      <c r="G102" s="130"/>
       <c r="M102" s="103"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="103"/>
-      <c r="B103" s="0" t="n">
-        <f aca="false">B102+1</f>
-        <v>92</v>
-      </c>
-      <c r="C103" s="30" t="s">
-        <v>562</v>
-      </c>
-      <c r="D103" s="30" t="s">
-        <v>563</v>
-      </c>
-      <c r="E103" s="111"/>
-      <c r="F103" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="G103" s="124"/>
-      <c r="H103" s="57"/>
-      <c r="I103" s="115"/>
-      <c r="J103" s="114" t="s">
-        <v>564</v>
-      </c>
-      <c r="K103" s="114"/>
       <c r="M103" s="103"/>
     </row>
-    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="103"/>
-      <c r="B104" s="0" t="n">
-        <f aca="false">B103+1</f>
-        <v>93</v>
-      </c>
-      <c r="C104" s="30" t="s">
-        <v>565</v>
-      </c>
-      <c r="D104" s="30" t="s">
-        <v>566</v>
-      </c>
-      <c r="E104" s="111"/>
-      <c r="F104" s="121" t="n">
-        <v>4</v>
-      </c>
-      <c r="G104" s="124"/>
-      <c r="H104" s="57" t="s">
-        <v>328</v>
-      </c>
-      <c r="I104" s="115"/>
-      <c r="J104" s="114" t="s">
-        <v>567</v>
-      </c>
-      <c r="K104" s="114" t="s">
-        <v>568</v>
-      </c>
+      <c r="C104" s="130" t="s">
+        <v>576</v>
+      </c>
+      <c r="D104" s="130"/>
+      <c r="E104" s="130"/>
+      <c r="F104" s="130"/>
+      <c r="G104" s="130"/>
       <c r="M104" s="103"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="103"/>
-      <c r="B105" s="0" t="n">
-        <f aca="false">B104+1</f>
-        <v>94</v>
-      </c>
-      <c r="C105" s="30" t="s">
-        <v>569</v>
-      </c>
-      <c r="D105" s="30" t="s">
-        <v>570</v>
-      </c>
-      <c r="E105" s="111"/>
-      <c r="F105" s="121" t="n">
-        <v>5</v>
-      </c>
-      <c r="G105" s="124"/>
-      <c r="H105" s="57"/>
-      <c r="I105" s="115"/>
-      <c r="J105" s="114" t="s">
-        <v>571</v>
-      </c>
-      <c r="K105" s="114"/>
       <c r="M105" s="103"/>
     </row>
-    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="103"/>
-      <c r="B106" s="0" t="n">
-        <f aca="false">B105+1</f>
-        <v>95</v>
-      </c>
-      <c r="C106" s="30" t="s">
-        <v>572</v>
-      </c>
-      <c r="D106" s="30" t="s">
-        <v>573</v>
-      </c>
-      <c r="E106" s="111"/>
-      <c r="F106" s="121" t="n">
-        <v>7</v>
-      </c>
-      <c r="G106" s="126"/>
-      <c r="H106" s="57"/>
-      <c r="I106" s="129"/>
-      <c r="J106" s="114" t="s">
-        <v>574</v>
-      </c>
-      <c r="K106" s="114" t="s">
-        <v>568</v>
-      </c>
+      <c r="C106" s="131" t="s">
+        <v>577</v>
+      </c>
+      <c r="D106" s="131"/>
+      <c r="E106" s="131"/>
+      <c r="F106" s="131"/>
+      <c r="G106" s="131"/>
+      <c r="H106" s="131"/>
       <c r="M106" s="103"/>
     </row>
-    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="103"/>
+      <c r="C107" s="110" t="s">
+        <v>578</v>
+      </c>
+      <c r="D107" s="132" t="s">
+        <v>579</v>
+      </c>
+      <c r="E107" s="132"/>
+      <c r="F107" s="132"/>
+      <c r="G107" s="132"/>
+      <c r="H107" s="132" t="s">
+        <v>580</v>
+      </c>
+      <c r="I107" s="132"/>
+      <c r="J107" s="132"/>
+      <c r="K107" s="132"/>
       <c r="M107" s="103"/>
     </row>
-    <row r="108" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="103"/>
-      <c r="C108" s="130" t="s">
-        <v>575</v>
-      </c>
-      <c r="D108" s="130"/>
-      <c r="E108" s="130"/>
-      <c r="F108" s="130"/>
-      <c r="G108" s="130"/>
+      <c r="C108" s="110" t="s">
+        <v>581</v>
+      </c>
+      <c r="D108" s="132" t="s">
+        <v>582</v>
+      </c>
+      <c r="E108" s="132"/>
+      <c r="F108" s="132"/>
+      <c r="G108" s="132"/>
+      <c r="H108" s="133" t="s">
+        <v>583</v>
+      </c>
+      <c r="I108" s="133"/>
+      <c r="J108" s="133"/>
+      <c r="K108" s="133"/>
       <c r="M108" s="103"/>
     </row>
-    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="103"/>
+      <c r="C109" s="110" t="s">
+        <v>584</v>
+      </c>
+      <c r="D109" s="132" t="s">
+        <v>585</v>
+      </c>
+      <c r="E109" s="132"/>
+      <c r="F109" s="132"/>
+      <c r="G109" s="132"/>
+      <c r="H109" s="132" t="s">
+        <v>586</v>
+      </c>
+      <c r="I109" s="132"/>
+      <c r="J109" s="132"/>
+      <c r="K109" s="132"/>
       <c r="M109" s="103"/>
     </row>
-    <row r="110" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="103"/>
-      <c r="C110" s="130" t="s">
-        <v>576</v>
-      </c>
-      <c r="D110" s="130"/>
-      <c r="E110" s="130"/>
-      <c r="F110" s="130"/>
-      <c r="G110" s="130"/>
+      <c r="C110" s="110" t="s">
+        <v>587</v>
+      </c>
+      <c r="D110" s="132" t="s">
+        <v>588</v>
+      </c>
+      <c r="E110" s="132"/>
+      <c r="F110" s="132"/>
+      <c r="G110" s="132"/>
+      <c r="H110" s="132" t="s">
+        <v>589</v>
+      </c>
+      <c r="I110" s="132"/>
+      <c r="J110" s="132"/>
+      <c r="K110" s="132"/>
       <c r="M110" s="103"/>
     </row>
-    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="103"/>
+      <c r="C111" s="110" t="s">
+        <v>590</v>
+      </c>
+      <c r="D111" s="132" t="s">
+        <v>591</v>
+      </c>
+      <c r="E111" s="132"/>
+      <c r="F111" s="132"/>
+      <c r="G111" s="132"/>
+      <c r="H111" s="132" t="s">
+        <v>592</v>
+      </c>
+      <c r="I111" s="132"/>
+      <c r="J111" s="132"/>
+      <c r="K111" s="132"/>
       <c r="M111" s="103"/>
     </row>
-    <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="103"/>
-      <c r="C112" s="131" t="s">
-        <v>577</v>
-      </c>
-      <c r="D112" s="131"/>
-      <c r="E112" s="131"/>
-      <c r="F112" s="131"/>
-      <c r="G112" s="131"/>
-      <c r="H112" s="131"/>
+      <c r="C112" s="134" t="s">
+        <v>593</v>
+      </c>
+      <c r="D112" s="134"/>
+      <c r="E112" s="134"/>
+      <c r="F112" s="134"/>
       <c r="M112" s="103"/>
     </row>
-    <row r="113" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="103"/>
-      <c r="C113" s="110" t="s">
-        <v>578</v>
-      </c>
-      <c r="D113" s="132" t="s">
-        <v>579</v>
-      </c>
-      <c r="E113" s="132"/>
-      <c r="F113" s="132"/>
-      <c r="G113" s="132"/>
-      <c r="H113" s="132" t="s">
-        <v>580</v>
-      </c>
-      <c r="I113" s="132"/>
-      <c r="J113" s="132"/>
-      <c r="K113" s="132"/>
+      <c r="C113" s="0" t="s">
+        <v>594</v>
+      </c>
       <c r="M113" s="103"/>
     </row>
-    <row r="114" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="103"/>
-      <c r="C114" s="110" t="s">
-        <v>581</v>
-      </c>
-      <c r="D114" s="132" t="s">
-        <v>582</v>
-      </c>
-      <c r="E114" s="132"/>
-      <c r="F114" s="132"/>
-      <c r="G114" s="132"/>
-      <c r="H114" s="133" t="s">
-        <v>583</v>
-      </c>
-      <c r="I114" s="133"/>
-      <c r="J114" s="133"/>
-      <c r="K114" s="133"/>
+      <c r="C114" s="0" t="s">
+        <v>595</v>
+      </c>
       <c r="M114" s="103"/>
     </row>
-    <row r="115" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="103"/>
-      <c r="C115" s="110" t="s">
-        <v>584</v>
-      </c>
-      <c r="D115" s="132" t="s">
-        <v>585</v>
-      </c>
-      <c r="E115" s="132"/>
-      <c r="F115" s="132"/>
-      <c r="G115" s="132"/>
-      <c r="H115" s="132" t="s">
-        <v>586</v>
-      </c>
-      <c r="I115" s="132"/>
-      <c r="J115" s="132"/>
-      <c r="K115" s="132"/>
+      <c r="C115" s="134" t="s">
+        <v>596</v>
+      </c>
+      <c r="D115" s="134"/>
+      <c r="E115" s="134"/>
+      <c r="F115" s="134"/>
       <c r="M115" s="103"/>
     </row>
-    <row r="116" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="103"/>
-      <c r="C116" s="110" t="s">
-        <v>587</v>
-      </c>
-      <c r="D116" s="132" t="s">
-        <v>588</v>
-      </c>
-      <c r="E116" s="132"/>
-      <c r="F116" s="132"/>
-      <c r="G116" s="132"/>
-      <c r="H116" s="132" t="s">
-        <v>589</v>
-      </c>
-      <c r="I116" s="132"/>
-      <c r="J116" s="132"/>
-      <c r="K116" s="132"/>
+      <c r="C116" s="0" t="s">
+        <v>597</v>
+      </c>
       <c r="M116" s="103"/>
     </row>
-    <row r="117" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="103"/>
-      <c r="C117" s="110" t="s">
-        <v>590</v>
-      </c>
-      <c r="D117" s="132" t="s">
-        <v>591</v>
-      </c>
-      <c r="E117" s="132"/>
-      <c r="F117" s="132"/>
-      <c r="G117" s="132"/>
-      <c r="H117" s="132" t="s">
-        <v>592</v>
-      </c>
-      <c r="I117" s="132"/>
-      <c r="J117" s="132"/>
-      <c r="K117" s="132"/>
+      <c r="B117" s="103"/>
+      <c r="C117" s="103"/>
+      <c r="D117" s="103"/>
+      <c r="E117" s="103"/>
+      <c r="F117" s="103"/>
+      <c r="G117" s="103"/>
+      <c r="H117" s="103"/>
+      <c r="I117" s="103"/>
+      <c r="J117" s="103"/>
+      <c r="K117" s="103"/>
+      <c r="L117" s="103"/>
       <c r="M117" s="103"/>
-    </row>
-    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="103"/>
-      <c r="C118" s="134" t="s">
-        <v>593</v>
-      </c>
-      <c r="D118" s="134"/>
-      <c r="E118" s="134"/>
-      <c r="F118" s="134"/>
-      <c r="M118" s="103"/>
-    </row>
-    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="103"/>
-      <c r="C119" s="0" t="s">
-        <v>594</v>
-      </c>
-      <c r="M119" s="103"/>
-    </row>
-    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="103"/>
-      <c r="C120" s="0" t="s">
-        <v>595</v>
-      </c>
-      <c r="M120" s="103"/>
-    </row>
-    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="103"/>
-      <c r="C121" s="134" t="s">
-        <v>596</v>
-      </c>
-      <c r="D121" s="134"/>
-      <c r="E121" s="134"/>
-      <c r="F121" s="134"/>
-      <c r="M121" s="103"/>
-    </row>
-    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="103"/>
-      <c r="C122" s="0" t="s">
-        <v>597</v>
-      </c>
-      <c r="M122" s="103"/>
-    </row>
-    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="103"/>
-      <c r="B123" s="103"/>
-      <c r="C123" s="103"/>
-      <c r="D123" s="103"/>
-      <c r="E123" s="103"/>
-      <c r="F123" s="103"/>
-      <c r="G123" s="103"/>
-      <c r="H123" s="103"/>
-      <c r="I123" s="103"/>
-      <c r="J123" s="103"/>
-      <c r="K123" s="103"/>
-      <c r="L123" s="103"/>
-      <c r="M123" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="91">
@@ -18100,33 +18010,33 @@
     <mergeCell ref="H63:H68"/>
     <mergeCell ref="G65:G66"/>
     <mergeCell ref="G67:G68"/>
-    <mergeCell ref="E69:E99"/>
-    <mergeCell ref="F69:F83"/>
+    <mergeCell ref="E69:E93"/>
+    <mergeCell ref="F69:F80"/>
     <mergeCell ref="H69:H73"/>
-    <mergeCell ref="H74:H79"/>
-    <mergeCell ref="H80:H83"/>
-    <mergeCell ref="F84:F99"/>
-    <mergeCell ref="H84:H89"/>
-    <mergeCell ref="H90:H95"/>
-    <mergeCell ref="H96:H99"/>
-    <mergeCell ref="E100:E106"/>
-    <mergeCell ref="H100:H103"/>
-    <mergeCell ref="H104:H106"/>
-    <mergeCell ref="C108:G108"/>
-    <mergeCell ref="C110:G110"/>
-    <mergeCell ref="C112:H112"/>
-    <mergeCell ref="D113:G113"/>
-    <mergeCell ref="H113:K113"/>
-    <mergeCell ref="D114:G114"/>
-    <mergeCell ref="H114:K114"/>
-    <mergeCell ref="D115:G115"/>
-    <mergeCell ref="H115:K115"/>
-    <mergeCell ref="D116:G116"/>
-    <mergeCell ref="H116:K116"/>
-    <mergeCell ref="D117:G117"/>
-    <mergeCell ref="H117:K117"/>
-    <mergeCell ref="C118:F118"/>
-    <mergeCell ref="C121:F121"/>
+    <mergeCell ref="H74:H76"/>
+    <mergeCell ref="H77:H80"/>
+    <mergeCell ref="F81:F93"/>
+    <mergeCell ref="H81:H86"/>
+    <mergeCell ref="H87:H89"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="E94:E100"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="H98:H100"/>
+    <mergeCell ref="C102:G102"/>
+    <mergeCell ref="C104:G104"/>
+    <mergeCell ref="C106:H106"/>
+    <mergeCell ref="D107:G107"/>
+    <mergeCell ref="H107:K107"/>
+    <mergeCell ref="D108:G108"/>
+    <mergeCell ref="H108:K108"/>
+    <mergeCell ref="D109:G109"/>
+    <mergeCell ref="H109:K109"/>
+    <mergeCell ref="D110:G110"/>
+    <mergeCell ref="H110:K110"/>
+    <mergeCell ref="D111:G111"/>
+    <mergeCell ref="H111:K111"/>
+    <mergeCell ref="C112:F112"/>
+    <mergeCell ref="C115:F115"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.511811023622047" footer="0.511811023622047"/>
@@ -33139,7 +33049,7 @@
       <c r="I314" s="57"/>
       <c r="J314" s="57"/>
       <c r="K314" s="228" t="s">
-        <v>1302</v>
+        <v>1332</v>
       </c>
       <c r="L314" s="228"/>
       <c r="M314" s="228"/>
@@ -33179,7 +33089,7 @@
       <c r="I315" s="57"/>
       <c r="J315" s="57"/>
       <c r="K315" s="228" t="s">
-        <v>1303</v>
+        <v>1333</v>
       </c>
       <c r="L315" s="228"/>
       <c r="M315" s="228"/>
@@ -33219,7 +33129,7 @@
       <c r="I316" s="57"/>
       <c r="J316" s="57"/>
       <c r="K316" s="228" t="s">
-        <v>1304</v>
+        <v>1334</v>
       </c>
       <c r="L316" s="228"/>
       <c r="M316" s="228"/>
@@ -33259,7 +33169,7 @@
       <c r="I317" s="57"/>
       <c r="J317" s="57"/>
       <c r="K317" s="228" t="s">
-        <v>1305</v>
+        <v>1335</v>
       </c>
       <c r="L317" s="228"/>
       <c r="M317" s="228"/>
@@ -33299,7 +33209,7 @@
       <c r="I318" s="57"/>
       <c r="J318" s="57"/>
       <c r="K318" s="228" t="s">
-        <v>1306</v>
+        <v>1336</v>
       </c>
       <c r="L318" s="228"/>
       <c r="M318" s="228"/>
@@ -33339,7 +33249,7 @@
       <c r="I319" s="57"/>
       <c r="J319" s="57"/>
       <c r="K319" s="228" t="s">
-        <v>1307</v>
+        <v>1337</v>
       </c>
       <c r="L319" s="228"/>
       <c r="M319" s="228"/>
@@ -33857,7 +33767,7 @@
       <c r="I332" s="95"/>
       <c r="J332" s="95"/>
       <c r="K332" s="228" t="s">
-        <v>1308</v>
+        <v>1338</v>
       </c>
       <c r="L332" s="228"/>
       <c r="M332" s="228"/>
@@ -33899,7 +33809,7 @@
       <c r="I333" s="95"/>
       <c r="J333" s="95"/>
       <c r="K333" s="228" t="s">
-        <v>1309</v>
+        <v>1339</v>
       </c>
       <c r="L333" s="228"/>
       <c r="M333" s="228"/>
@@ -33938,7 +33848,7 @@
       <c r="I334" s="95"/>
       <c r="J334" s="95"/>
       <c r="K334" s="228" t="s">
-        <v>1310</v>
+        <v>1340</v>
       </c>
       <c r="L334" s="228"/>
       <c r="M334" s="228"/>
@@ -33977,7 +33887,7 @@
       <c r="I335" s="95"/>
       <c r="J335" s="95"/>
       <c r="K335" s="228" t="s">
-        <v>1311</v>
+        <v>1341</v>
       </c>
       <c r="L335" s="228"/>
       <c r="M335" s="228"/>
@@ -34016,7 +33926,7 @@
       <c r="I336" s="95"/>
       <c r="J336" s="95"/>
       <c r="K336" s="228" t="s">
-        <v>1312</v>
+        <v>1342</v>
       </c>
       <c r="L336" s="228"/>
       <c r="M336" s="228"/>
@@ -34055,7 +33965,7 @@
       <c r="I337" s="95"/>
       <c r="J337" s="95"/>
       <c r="K337" s="228" t="s">
-        <v>1313</v>
+        <v>1343</v>
       </c>
       <c r="L337" s="228"/>
       <c r="M337" s="228"/>

</xml_diff>

<commit_message>
Still adding a 65C64 simulator.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="1344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="1376">
   <si>
     <t xml:space="preserve">Pin number</t>
   </si>
@@ -6112,6 +6112,102 @@
   </si>
   <si>
     <t xml:space="preserve">11 = Unused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">![W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ∧[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ∧[W]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ∨[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ⊻[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] + [W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] - [W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] - [W]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load [W] into DI.  Load [V] into DJ.  z set indicates DJ was 0.  n indicates DJ was negative.  Store DI into [V].   Increment V, Increment W, decrement A.  v set indicates A is negative after decrement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ∧[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ∨[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V] ⊻[W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[V]; [W] → [V]; A-1 → A; V+o → V; W+o → W; {C+i → C}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V is the source address; A is the destination address; W is the number of bytes to copy (a multiple of 8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The loop copies from offset W down to offset 8 (z is set when W reaches 0), so V and A start 8 below the source and destination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wth A, 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embedded 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set A width to 4 bytes (A holds the destination address)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pul (A, V, W), S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pull using stack S into registers in order W, V, A.  1 + 2 words each (S aligned)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpy B, V+W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy into B the 64 bit value in address V+W.  1 + 4 words</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpy A+W, B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy B into address A+W.  1 + 4 words</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copies 8 bytes in 12 cycles (5 + 5 + 1 + 1, aligned, 16 bit data bus): 1.50 cycles per byte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W is the source address; V is the destination address; A + 1 is the number of 64 bit values to copy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pull using stack S into registers in order W, V, A.  1 + 2 words each (S aligned)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy the 64 bit value in address W into address V.  Increment W by 8.  Increment V by 8.  Decrement A by 1.  v is set when A is negative; vcpy repeats until then.  1 + 4 reads + 4 writes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copies 8 bytes in 9 cycles (aligned, 16 bit data bus): 1.13 cycles per byte</t>
   </si>
 </sst>
 </file>
@@ -9125,7 +9221,7 @@
       <c r="F2" s="107"/>
       <c r="G2" s="107"/>
       <c r="H2" s="102" t="s">
-        <v>1079</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9136,7 +9232,7 @@
       <c r="F3" s="107"/>
       <c r="G3" s="107"/>
       <c r="H3" s="102" t="s">
-        <v>1080</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9154,22 +9250,22 @@
         <v>0</v>
       </c>
       <c r="C5" s="127" t="s">
-        <v>1082</v>
+        <v>1361</v>
       </c>
       <c r="D5" s="102" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="102" t="s">
-        <v>1083</v>
+        <v>1362</v>
       </c>
       <c r="F5" s="102" t="s">
-        <v>1084</v>
+        <v>1363</v>
       </c>
       <c r="G5" s="102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="102" t="s">
-        <v>1085</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9191,7 +9287,7 @@
         <v>1089</v>
       </c>
       <c r="G6" s="102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="102" t="s">
         <v>1090</v>
@@ -9204,7 +9300,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="255" t="s">
-        <v>1091</v>
+        <v>1365</v>
       </c>
       <c r="D7" s="102" t="n">
         <v>2</v>
@@ -9215,11 +9311,11 @@
       <c r="F7" s="102" t="s">
         <v>1083</v>
       </c>
-      <c r="G7" s="102" t="s">
-        <v>1092</v>
+      <c r="G7" s="102" t="n">
+        <v>7</v>
       </c>
       <c r="H7" s="102" t="s">
-        <v>1093</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9236,7 +9332,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="127" t="s">
-        <v>1095</v>
+        <v>1367</v>
       </c>
       <c r="D9" s="102" t="s">
         <v>1096</v>
@@ -9247,11 +9343,11 @@
       <c r="F9" s="0" t="s">
         <v>960</v>
       </c>
-      <c r="G9" s="102" t="s">
-        <v>1097</v>
+      <c r="G9" s="102" t="n">
+        <v>5</v>
       </c>
       <c r="H9" s="102" t="s">
-        <v>1316</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9261,7 +9357,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="127" t="s">
-        <v>1099</v>
+        <v>1369</v>
       </c>
       <c r="D10" s="102" t="s">
         <v>1096</v>
@@ -9272,11 +9368,11 @@
       <c r="F10" s="0" t="s">
         <v>960</v>
       </c>
-      <c r="G10" s="102" t="s">
-        <v>1097</v>
+      <c r="G10" s="102" t="n">
+        <v>5</v>
       </c>
       <c r="H10" s="102" t="s">
-        <v>1100</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9341,7 +9437,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="119" t="s">
-        <v>1107</v>
+        <v>1371</v>
       </c>
       <c r="B14" s="119"/>
       <c r="C14" s="119"/>
@@ -9353,7 +9449,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H16" s="102" t="s">
-        <v>1108</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9382,7 +9478,7 @@
         <v>1084</v>
       </c>
       <c r="G18" s="102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9404,7 +9500,7 @@
         <v>1318</v>
       </c>
       <c r="G19" s="102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,8 +9521,11 @@
       <c r="F20" s="102" t="s">
         <v>1083</v>
       </c>
-      <c r="G20" s="102" t="s">
-        <v>1111</v>
+      <c r="G20" s="102" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" s="102" t="s">
+        <v>1373</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9450,11 +9549,11 @@
       <c r="E22" s="102" t="s">
         <v>1113</v>
       </c>
-      <c r="G22" s="102" t="s">
-        <v>1097</v>
+      <c r="G22" s="102" t="n">
+        <v>9</v>
       </c>
       <c r="H22" s="102" t="s">
-        <v>1114</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9469,7 +9568,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="119" t="s">
-        <v>1115</v>
+        <v>1375</v>
       </c>
       <c r="B24" s="119"/>
       <c r="C24" s="119"/>
@@ -17215,7 +17314,7 @@
       </c>
       <c r="I81" s="115"/>
       <c r="J81" s="114" t="s">
-        <v>513</v>
+        <v>1344</v>
       </c>
       <c r="K81" s="114" t="s">
         <v>471</v>
@@ -17245,7 +17344,7 @@
       <c r="H82" s="125"/>
       <c r="I82" s="127"/>
       <c r="J82" s="114" t="s">
-        <v>517</v>
+        <v>1345</v>
       </c>
       <c r="K82" s="114" t="s">
         <v>471</v>
@@ -17275,7 +17374,7 @@
       <c r="H83" s="125"/>
       <c r="I83" s="115"/>
       <c r="J83" s="114" t="s">
-        <v>521</v>
+        <v>1346</v>
       </c>
       <c r="K83" s="114" t="s">
         <v>471</v>
@@ -17305,7 +17404,7 @@
       <c r="H84" s="125"/>
       <c r="I84" s="115"/>
       <c r="J84" s="114" t="s">
-        <v>1274</v>
+        <v>1347</v>
       </c>
       <c r="K84" s="114" t="s">
         <v>471</v>
@@ -17332,7 +17431,7 @@
       <c r="H85" s="125"/>
       <c r="I85" s="115"/>
       <c r="J85" s="114" t="s">
-        <v>1275</v>
+        <v>1348</v>
       </c>
       <c r="K85" s="114" t="s">
         <v>471</v>
@@ -17359,7 +17458,7 @@
       <c r="H86" s="125"/>
       <c r="I86" s="115"/>
       <c r="J86" s="114" t="s">
-        <v>1276</v>
+        <v>1349</v>
       </c>
       <c r="K86" s="114" t="s">
         <v>471</v>
@@ -17388,7 +17487,7 @@
       </c>
       <c r="I87" s="115"/>
       <c r="J87" s="114" t="s">
-        <v>1277</v>
+        <v>1350</v>
       </c>
       <c r="K87" s="114" t="s">
         <v>471</v>
@@ -17415,7 +17514,7 @@
       <c r="H88" s="125"/>
       <c r="I88" s="115"/>
       <c r="J88" s="114" t="s">
-        <v>1279</v>
+        <v>1351</v>
       </c>
       <c r="K88" s="114" t="s">
         <v>471</v>
@@ -17442,7 +17541,7 @@
       <c r="H89" s="125"/>
       <c r="I89" s="115"/>
       <c r="J89" s="114" t="s">
-        <v>538</v>
+        <v>1352</v>
       </c>
       <c r="K89" s="114" t="s">
         <v>471</v>
@@ -17471,13 +17570,13 @@
       </c>
       <c r="I90" s="115"/>
       <c r="J90" s="114" t="s">
-        <v>513</v>
+        <v>1358</v>
       </c>
       <c r="K90" s="114" t="s">
         <v>471</v>
       </c>
       <c r="L90" s="0" t="s">
-        <v>514</v>
+        <v>1354</v>
       </c>
       <c r="M90" s="103"/>
     </row>
@@ -17501,7 +17600,7 @@
       <c r="H91" s="125"/>
       <c r="I91" s="115"/>
       <c r="J91" s="114" t="s">
-        <v>521</v>
+        <v>1355</v>
       </c>
       <c r="K91" s="114" t="s">
         <v>471</v>
@@ -17528,7 +17627,7 @@
       <c r="H92" s="125"/>
       <c r="I92" s="115"/>
       <c r="J92" s="114" t="s">
-        <v>1281</v>
+        <v>1356</v>
       </c>
       <c r="K92" s="114" t="s">
         <v>471</v>
@@ -17555,7 +17654,7 @@
       <c r="H93" s="125"/>
       <c r="I93" s="115"/>
       <c r="J93" s="114" t="s">
-        <v>1282</v>
+        <v>1357</v>
       </c>
       <c r="K93" s="114" t="s">
         <v>471</v>

</xml_diff>

<commit_message>
Update 65C64 Instruction Architecture to reflect what the simulator actually does.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="1376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2618" uniqueCount="1413">
   <si>
     <t xml:space="preserve">Pin number</t>
   </si>
@@ -2881,7 +2881,7 @@
     <t xml:space="preserve">v, z, c</t>
   </si>
   <si>
-    <t xml:space="preserve">W must be assigned 0 initially.  A is the divisor, B is the quotient.  Y contains the dividend and W the remainder when v is set.   Repeat partial divide whilst v is not set.  z set indicates Y is zero.  c clear indicates W is zero.</t>
+    <t xml:space="preserve">W must be assigned 0 initially.  A is the divisor and Y the dividend.  B is the top half of the dividend: usually 0, but any value below A divides B and Y together, (B &lt;&lt; Y’s width) + Y.  Y contains the quotient and B the remainder when v is set.   Repeat partial divide whilst v is not set.  z set indicates Y is zero.  c clear indicates B is zero.</t>
   </si>
   <si>
     <t xml:space="preserve">Negate</t>
@@ -6209,6 +6209,117 @@
   <si>
     <t xml:space="preserve">Copies 8 bytes in 9 cycles (aligned, 16 bit data bus): 1.13 cycles per byte</t>
   </si>
+  <si>
+    <t xml:space="preserve">Sign or zero extension only applies to the second operand, when it is narrower than the operation (the width of the register operand, or 32 bits without one).  The first operand is never extended.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 ∧ O2:s → O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 ∨ O2:s → O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 ⊻ O2:s → O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 ∧ O2:s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 + O2:s → O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 - O2:s → O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n, v, z, c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v is set as by subtract (and c is not borrow), so a signed comparison can branch on n ≠ v (braso (n, v)).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O1 - O2:s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n, v, z, c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copies bytes from the index in the first register to the second register for count bytes, index incrementing.  Subcopy ignores the set width of a register.    Source bytes past 63 read as 0 and destination bytes past 63 are dropped.  n and z are set from the second register at its width.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copies bits from index in first register to second register for count bits, index incrementing.  Subcopy ignores the set width of a register.    Source bits past 63 read as 0 and destination bits past 63 are dropped.  n and z are set from the second register at its width.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{P → [S]; S-2 → S}; O2 → C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+i → C; {P → [S]; S-2 → S}; C + O2 → C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtracts 1 from the interrupt depth.  e and l come back with P.  The stack can be S, V, W or Y.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+i → C; C → [S]; S-4 → S; P → [S]; S-2 → S; [vector] → C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector n (0 to 1023) is at FFFF:F000 + 4n.  Adds 1 to the interrupt depth.  Unlike an interrupt, brk leaves e and l as they are.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Without wake bits the processor stops until reset.  With wake bits (l, e0 to e3) it waits for one of those interrupts, even a disabled one: an enabled interrupt is taken (with C after stp), a disabled one continues after stp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8r → R; {8r - 1 → R}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The width in bits, or one less with gwth R, (Q, -1) (see the ror example).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c is set to O1:b[o1] after shifting.  v is set to O1:b[o1+1] after shifting.  A shift of 0 clears c and v.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c is set to O1:b[-1] after shifting.  v is set to O1:b[-2] after shifting.  n is set to O1:b[o1-1] before shifting.  A shift of 0 clears c and v.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pushed in the order A, B, S, V, W, X, Y, each at its width, with the values from before the stack register moves.  n and z are set from the last register pushed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulled in the order Y, X, W, V, S, B, A (the reverse), each at its width.  n and z are set from the last register pulled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An immediate is pushed at its own width; the value at an address is pushed as 32 bits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Always pulls 32 bits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W must be assigned 0 initially.  A and B are multiplicands.  Y contains the result when v is set.   Repeat partial multiply whilst v is not set. z set indicates Y is zero.  W counts B’s nybbles, two a step, so there is a step for each byte of B.  The first step clears Y, and the product is truncated to Y’s width.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W must be assigned 0 initially.  A is the divisor and Y the dividend.  B is the top half of the dividend: usually 0, but any value below A divides B and Y together, (B &lt;&lt; Y’s width) + Y.  Y contains the quotient and B the remainder when v is set.   Repeat partial divide whilst v is not set.  z set indicates Y is zero.  c clear indicates B is zero.  W counts Y’s nybbles, one a step.  The remainder is truncated to B’s width every step.  Dividing by 0 gives quotient nybbles of 15.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 - R2:s → R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abs(R2:s) → R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scan first register from bit indexed by count register in direction until bit in first is high.  Pre-increment count if c set.  v set indicates no more bits.  c is always set.  When nothing is found the count is one past the end: the width in units going up, all ones going down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store R into [V].   Increment V, decrement A.  v set indicates A is negative after decrement.  It never stops early (its stop bits are ignored).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load [V] into D.  And D with R.  Store D into [V].  Increment V, decrement A.  v set indicates A is negative after decrement.  z set indicates D was 0.  n indicates D was negative.  Every block and vector operation but bcpy repeats (C stays on the opcode) until v is set or, if stopping is allowed, its stop condition (z set, z clear, n set or n clear) holds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load [W] into D.  Store D into [V].   Increment V, Increment W, decrement A.  v set indicates A is negative after decrement.  z set indicates D was 0.  n indicates D was negative.  Like the block operations, it repeats until v is set or an allowed stop condition holds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p → R:b[N]; {p → R:b[N±1] … R:b[N±(count-1)]}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With a repeat the flag is written to count bits (a register, or 0 to 63) from bit N up or down.  Bits outside 0 to 63 are dropped and the register’s width is ignored; 32 or more bits take a cycle more.</t>
+  </si>
 </sst>
 </file>
 
@@ -6221,7 +6332,7 @@
     <numFmt numFmtId="167" formatCode="#,###.0"/>
     <numFmt numFmtId="168" formatCode="#,###"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -6330,6 +6441,12 @@
       <color rgb="FFCCCCCC"/>
       <name val="Courier New"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="24">
@@ -6689,7 +6806,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="269">
+  <cellXfs count="272">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7766,6 +7883,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15319,6 +15448,9 @@
       <c r="K12" s="114" t="s">
         <v>254</v>
       </c>
+      <c r="L12" s="269" t="s">
+        <v>1376</v>
+      </c>
       <c r="M12" s="103"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15369,8 +15501,8 @@
       </c>
       <c r="H14" s="57"/>
       <c r="I14" s="115"/>
-      <c r="J14" s="114" t="s">
-        <v>261</v>
+      <c r="J14" s="270" t="s">
+        <v>1377</v>
       </c>
       <c r="K14" s="114" t="s">
         <v>254</v>
@@ -15425,8 +15557,8 @@
       </c>
       <c r="H16" s="57"/>
       <c r="I16" s="115"/>
-      <c r="J16" s="114" t="s">
-        <v>267</v>
+      <c r="J16" s="270" t="s">
+        <v>1378</v>
       </c>
       <c r="K16" s="114" t="s">
         <v>254</v>
@@ -15481,8 +15613,8 @@
       </c>
       <c r="H18" s="57"/>
       <c r="I18" s="115"/>
-      <c r="J18" s="114" t="s">
-        <v>1270</v>
+      <c r="J18" s="270" t="s">
+        <v>1379</v>
       </c>
       <c r="K18" s="114" t="s">
         <v>254</v>
@@ -15537,8 +15669,8 @@
       </c>
       <c r="H20" s="57"/>
       <c r="I20" s="115"/>
-      <c r="J20" s="114" t="s">
-        <v>1271</v>
+      <c r="J20" s="270" t="s">
+        <v>1380</v>
       </c>
       <c r="K20" s="114" t="s">
         <v>254</v>
@@ -15595,8 +15727,8 @@
       </c>
       <c r="H22" s="57"/>
       <c r="I22" s="115"/>
-      <c r="J22" s="114" t="s">
-        <v>287</v>
+      <c r="J22" s="270" t="s">
+        <v>1381</v>
       </c>
       <c r="K22" s="114" t="s">
         <v>285</v>
@@ -15651,8 +15783,8 @@
       </c>
       <c r="H24" s="57"/>
       <c r="I24" s="115"/>
-      <c r="J24" s="114" t="s">
-        <v>1272</v>
+      <c r="J24" s="270" t="s">
+        <v>1382</v>
       </c>
       <c r="K24" s="114" t="s">
         <v>285</v>
@@ -15685,8 +15817,11 @@
       <c r="J25" s="114" t="s">
         <v>297</v>
       </c>
-      <c r="K25" s="114" t="s">
-        <v>298</v>
+      <c r="K25" s="270" t="s">
+        <v>1383</v>
+      </c>
+      <c r="L25" s="269" t="s">
+        <v>1384</v>
       </c>
       <c r="M25" s="103"/>
     </row>
@@ -15707,11 +15842,11 @@
       </c>
       <c r="H26" s="57"/>
       <c r="I26" s="115"/>
-      <c r="J26" s="114" t="s">
-        <v>1273</v>
-      </c>
-      <c r="K26" s="114" t="s">
-        <v>298</v>
+      <c r="J26" s="270" t="s">
+        <v>1385</v>
+      </c>
+      <c r="K26" s="270" t="s">
+        <v>1386</v>
       </c>
       <c r="M26" s="103"/>
     </row>
@@ -15746,8 +15881,8 @@
       <c r="K27" s="118" t="s">
         <v>254</v>
       </c>
-      <c r="L27" s="119" t="s">
-        <v>305</v>
+      <c r="L27" s="271" t="s">
+        <v>1387</v>
       </c>
       <c r="M27" s="103"/>
     </row>
@@ -15798,8 +15933,8 @@
       <c r="K29" s="114" t="s">
         <v>254</v>
       </c>
-      <c r="L29" s="0" t="s">
-        <v>310</v>
+      <c r="L29" s="269" t="s">
+        <v>1388</v>
       </c>
       <c r="M29" s="103"/>
     </row>
@@ -15828,8 +15963,8 @@
       <c r="I30" s="115" t="s">
         <v>312</v>
       </c>
-      <c r="J30" s="114" t="s">
-        <v>314</v>
+      <c r="J30" s="270" t="s">
+        <v>1389</v>
       </c>
       <c r="K30" s="114"/>
       <c r="M30" s="103"/>
@@ -15881,8 +16016,8 @@
       </c>
       <c r="H32" s="57"/>
       <c r="I32" s="115"/>
-      <c r="J32" s="114" t="s">
-        <v>321</v>
+      <c r="J32" s="270" t="s">
+        <v>1390</v>
       </c>
       <c r="K32" s="114"/>
       <c r="L32" s="0" t="s">
@@ -16056,6 +16191,9 @@
       <c r="K38" s="114" t="s">
         <v>337</v>
       </c>
+      <c r="L38" s="269" t="s">
+        <v>1391</v>
+      </c>
       <c r="M38" s="103"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16199,10 +16337,13 @@
       <c r="I43" s="115" t="s">
         <v>364</v>
       </c>
-      <c r="J43" s="114" t="s">
-        <v>365</v>
+      <c r="J43" s="270" t="s">
+        <v>1392</v>
       </c>
       <c r="K43" s="114"/>
+      <c r="L43" s="269" t="s">
+        <v>1393</v>
+      </c>
       <c r="M43" s="103"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16232,6 +16373,9 @@
         <v>369</v>
       </c>
       <c r="K44" s="114"/>
+      <c r="L44" s="269" t="s">
+        <v>1394</v>
+      </c>
       <c r="M44" s="103"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16255,10 +16399,13 @@
         <v>328</v>
       </c>
       <c r="I45" s="115"/>
-      <c r="J45" s="114" t="s">
-        <v>372</v>
+      <c r="J45" s="270" t="s">
+        <v>1395</v>
       </c>
       <c r="K45" s="114"/>
+      <c r="L45" s="269" t="s">
+        <v>1396</v>
+      </c>
       <c r="M45" s="103"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16479,8 +16626,8 @@
       <c r="K53" s="114" t="s">
         <v>400</v>
       </c>
-      <c r="L53" s="0" t="s">
-        <v>401</v>
+      <c r="L53" s="269" t="s">
+        <v>1397</v>
       </c>
       <c r="M53" s="103"/>
     </row>
@@ -16511,8 +16658,8 @@
       <c r="K54" s="114" t="s">
         <v>406</v>
       </c>
-      <c r="L54" s="0" t="s">
-        <v>407</v>
+      <c r="L54" s="269" t="s">
+        <v>1398</v>
       </c>
       <c r="M54" s="103"/>
     </row>
@@ -16547,6 +16694,9 @@
       <c r="K55" s="114" t="s">
         <v>254</v>
       </c>
+      <c r="L55" s="269" t="s">
+        <v>1399</v>
+      </c>
       <c r="M55" s="103"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16576,6 +16726,9 @@
       <c r="K56" s="114" t="s">
         <v>254</v>
       </c>
+      <c r="L56" s="269" t="s">
+        <v>1400</v>
+      </c>
       <c r="M56" s="103"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16605,6 +16758,9 @@
         <v>417</v>
       </c>
       <c r="K57" s="114"/>
+      <c r="L57" s="269" t="s">
+        <v>1401</v>
+      </c>
       <c r="M57" s="103"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16630,6 +16786,9 @@
         <v>419</v>
       </c>
       <c r="K58" s="114"/>
+      <c r="L58" s="269" t="s">
+        <v>1402</v>
+      </c>
       <c r="M58" s="103"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16663,8 +16822,8 @@
       <c r="K59" s="114" t="s">
         <v>424</v>
       </c>
-      <c r="L59" s="0" t="s">
-        <v>425</v>
+      <c r="L59" s="269" t="s">
+        <v>1403</v>
       </c>
       <c r="M59" s="103"/>
     </row>
@@ -16693,8 +16852,8 @@
       <c r="K60" s="114" t="s">
         <v>429</v>
       </c>
-      <c r="L60" s="0" t="s">
-        <v>430</v>
+      <c r="L60" s="269" t="s">
+        <v>1404</v>
       </c>
       <c r="M60" s="103"/>
     </row>
@@ -16719,8 +16878,8 @@
         <v>282</v>
       </c>
       <c r="I61" s="115"/>
-      <c r="J61" s="114" t="s">
-        <v>433</v>
+      <c r="J61" s="270" t="s">
+        <v>1405</v>
       </c>
       <c r="K61" s="114" t="s">
         <v>254</v>
@@ -16746,8 +16905,8 @@
       </c>
       <c r="H62" s="57"/>
       <c r="I62" s="115"/>
-      <c r="J62" s="114" t="s">
-        <v>436</v>
+      <c r="J62" s="270" t="s">
+        <v>1406</v>
       </c>
       <c r="K62" s="114" t="s">
         <v>254</v>
@@ -16786,8 +16945,8 @@
       <c r="K63" s="114" t="s">
         <v>441</v>
       </c>
-      <c r="L63" s="0" t="s">
-        <v>442</v>
+      <c r="L63" s="269" t="s">
+        <v>1407</v>
       </c>
       <c r="M63" s="103"/>
     </row>
@@ -16966,8 +17125,8 @@
       <c r="K69" s="114" t="s">
         <v>184</v>
       </c>
-      <c r="L69" s="0" t="s">
-        <v>467</v>
+      <c r="L69" s="269" t="s">
+        <v>1408</v>
       </c>
       <c r="M69" s="103"/>
     </row>
@@ -16996,8 +17155,8 @@
       <c r="K70" s="114" t="s">
         <v>471</v>
       </c>
-      <c r="L70" s="0" t="s">
-        <v>472</v>
+      <c r="L70" s="269" t="s">
+        <v>1409</v>
       </c>
       <c r="M70" s="103"/>
     </row>
@@ -17319,8 +17478,8 @@
       <c r="K81" s="114" t="s">
         <v>471</v>
       </c>
-      <c r="L81" s="0" t="s">
-        <v>514</v>
+      <c r="L81" s="269" t="s">
+        <v>1410</v>
       </c>
       <c r="M81" s="103"/>
     </row>
@@ -17813,10 +17972,13 @@
       <c r="G99" s="124"/>
       <c r="H99" s="57"/>
       <c r="I99" s="115"/>
-      <c r="J99" s="114" t="s">
-        <v>571</v>
+      <c r="J99" s="270" t="s">
+        <v>1411</v>
       </c>
       <c r="K99" s="114"/>
+      <c r="L99" s="269" t="s">
+        <v>1412</v>
+      </c>
       <c r="M99" s="103"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Change wth instruction specifier to bits.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -5274,7 +5274,7 @@
     <t xml:space="preserve">Setup:</t>
   </si>
   <si>
-    <t xml:space="preserve">wtth (X, Y), 4</t>
+    <t xml:space="preserve">wtth (X, Y), 32</t>
   </si>
   <si>
     <t xml:space="preserve">Multi Register</t>
@@ -5289,16 +5289,16 @@
     <t xml:space="preserve">wth W, 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Set B width to 4 bytes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wth B, 8</t>
+    <t xml:space="preserve">Set B width to 32 bits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wth B, 64</t>
   </si>
   <si>
     <t xml:space="preserve">Embedded 8</t>
   </si>
   <si>
-    <t xml:space="preserve">Set B width to 8 bytes</t>
+    <t xml:space="preserve">Set B width to 64 bits</t>
   </si>
   <si>
     <t xml:space="preserve">pul (W, X, Y), S</t>
@@ -5355,7 +5355,7 @@
     <t xml:space="preserve">W is the source address; V is the destination address; A is the number of iterations.</t>
   </si>
   <si>
-    <t xml:space="preserve">wth A, 4</t>
+    <t xml:space="preserve">wth A, 32</t>
   </si>
   <si>
     <t xml:space="preserve">pul (A, X, Y), S</t>
@@ -6165,7 +6165,7 @@
     <t xml:space="preserve">The loop copies from offset W down to offset 8 (z is set when W reaches 0), so V and A start 8 below the source and destination</t>
   </si>
   <si>
-    <t xml:space="preserve">wth A, 4</t>
+    <t xml:space="preserve">wth A, 32</t>
   </si>
   <si>
     <t xml:space="preserve">Register</t>
@@ -6174,7 +6174,7 @@
     <t xml:space="preserve">Embedded 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Set A width to 4 bytes (A holds the destination address)</t>
+    <t xml:space="preserve">Set A width to 32 bits (A holds the destination address)</t>
   </si>
   <si>
     <t xml:space="preserve">pul (A, V, W), S</t>

</xml_diff>

<commit_message>
Added a signed copy instruction.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -3791,7 +3791,7 @@
     <t xml:space="preserve">O2:o:s → R</t>
   </si>
   <si>
-    <t xml:space="preserve">Copy a value of a given width in memory into a register sign extended.  A value wider than the register is truncated.  n and z are set from the value copied.  The zero extending copy (and the copy into memory) is code 12 extend 3; there is no room for this one there.</t>
+    <t xml:space="preserve">Copy a value of a given width (8, 16 or 32 bits) in memory into a register sign extended.  A value wider than the register is truncated.  n and z are set from the value copied.  There is no sign extending copy into memory; use the zero extending cpyx.</t>
   </si>
   <si>
     <t xml:space="preserve">Status to status</t>
@@ -4738,7 +4738,7 @@
     <t xml:space="preserve">Hardware Register Index</t>
   </si>
   <si>
-    <t xml:space="preserve">Hardware, State, Copy Extend (sign extend)</t>
+    <t xml:space="preserve">Hardware, State, Copy Extend</t>
   </si>
   <si>
     <t xml:space="preserve">0 – 63</t>

</xml_diff>

<commit_message>
Code generator uses new cpyx instruction.
</commit_message>
<xml_diff>
--- a/W65C64/65C64 Instruction Architecture.xlsx
+++ b/W65C64/65C64 Instruction Architecture.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2655" uniqueCount="1296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2655" uniqueCount="1297">
   <si>
     <t xml:space="preserve">Pin number</t>
   </si>
@@ -6057,6 +6057,9 @@
   </si>
   <si>
     <t xml:space="preserve">r2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None, V, X or Y</t>
   </si>
 </sst>
 </file>
@@ -21475,7 +21478,7 @@
       <c r="G44" s="164"/>
       <c r="H44" s="164"/>
       <c r="I44" s="161" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="J44" s="161"/>
       <c r="K44" s="161" t="s">
@@ -21657,7 +21660,7 @@
       <c r="G48" s="169"/>
       <c r="H48" s="169"/>
       <c r="I48" s="178" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="J48" s="178"/>
       <c r="K48" s="58" t="s">
@@ -27913,7 +27916,7 @@
       </c>
       <c r="F189" s="58"/>
       <c r="G189" s="161" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="H189" s="161"/>
       <c r="I189" s="161" t="s">
@@ -28085,7 +28088,7 @@
       </c>
       <c r="F193" s="161"/>
       <c r="G193" s="58" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="H193" s="58"/>
       <c r="I193" s="58" t="s">
@@ -31609,7 +31612,7 @@
       </c>
       <c r="E275" s="58"/>
       <c r="F275" s="161" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="G275" s="161"/>
       <c r="H275" s="161" t="s">
@@ -32728,7 +32731,7 @@
       </c>
       <c r="G300" s="58"/>
       <c r="H300" s="161" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="I300" s="161"/>
       <c r="J300" s="161" t="s">
@@ -32908,7 +32911,7 @@
       </c>
       <c r="G304" s="183"/>
       <c r="H304" s="58" t="s">
-        <v>735</v>
+        <v>1296</v>
       </c>
       <c r="I304" s="58"/>
       <c r="J304" s="58" t="s">

</xml_diff>